<commit_message>
Stage 8 review fixes: E-007
</commit_message>
<xml_diff>
--- a/output/archive/WestravelleData/Stability/PV30/WA-2021-270/Results/Approved/PV30_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
+++ b/output/archive/WestravelleData/Stability/PV30/WA-2021-270/Results/Approved/PV30_PULLS_AND_SUITABILITY_RESULTS_Rev03.xlsx
@@ -33,6 +33,10 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00000000"/>
     </font>
     <font>
@@ -51,10 +55,6 @@
       <name val="Arial"/>
       <i val="1"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -87,14 +87,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -472,190 +472,197 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WA/2021/270 PV30 pulls and suitability results</t>
+          <t>Westravelle Analytical Ltd, a Tarnovell company</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>WA/2021/270 PV30 pulls and suitability results</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>WA/2021/270</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>LIMS</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>WST-21-008374</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Parvessune Pharmaceuticals</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Lead</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Alice Penrose</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Sequence owner</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Leon Wu</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Method validation</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Saira Mahmood</t>
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>30/09/2021</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Interim review (6 months)</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>31/03/2022</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Completion (12 months)</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>30/09/2022</t>
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Stability result</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Initial assay (% label claim)</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B16" s="4" t="n">
         <v>100.2</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Last timepoint (months)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B17" s="4" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Overall outcome</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Complies at all conditions and timepoints; no OOS or OOT results</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>All reported results comply. This table does not establish an OOT assessment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Reviewed by</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Alice Penrose</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Checked 30/09/2022</t>
         </is>
@@ -690,610 +697,610 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ICH chamber programme: pulls and results</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Assay as % label claim, impurities as % area. Water by Karl Fischer, % w/w. Result per protocol acceptance criteria.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Assay as % label claim, impurities as % area. Water by Karl Fischer, % w/w. Result per protocol acceptance criteria. Time zero is one initial analysis shared by all storage conditions; repeated initial rows do not represent separate pulls.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Timepoint (months)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Assay (% LC)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Imp A RRT 0.86 (%)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Imp B RRT 1.12 (%)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Total impurities (%)</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Water KF (% w/w)</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="6" t="n">
         <v>100.2</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="3" t="n">
         <v>0.05</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="7" t="n">
         <v>0.17</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="6" t="n">
         <v>99.8</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="7" t="n">
         <v>0.23</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="7" t="n">
         <v>1.2</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="6" t="n">
         <v>100.1</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="3" t="n">
         <v>0.08</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="7" t="n">
         <v>0.23</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="7" t="n">
         <v>2.4</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="6" t="n">
         <v>99.7</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="3" t="n">
         <v>0.11</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="7" t="n">
         <v>0.25</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="7" t="n">
         <v>1.9</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="6" t="n">
         <v>100.6</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="3" t="n">
         <v>0.13</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>0.06</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="7" t="n">
         <v>0.27</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="7" t="n">
         <v>2.3</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>25 °C/60% RH</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="3" t="n">
         <v>0.14</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>0.09</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="7" t="n">
         <v>0.28</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G10" s="7" t="n">
         <v>2.5</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="6" t="n">
         <v>100.2</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="3" t="n">
         <v>0.05</v>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="7" t="n">
         <v>0.17</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="6" t="n">
         <v>100.2</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="3" t="n">
         <v>0.06</v>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="7" t="n">
         <v>0.15</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="6" t="n">
         <v>100.1</v>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="3" t="n">
         <v>0.05</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="7" t="n">
         <v>0.23</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="7" t="n">
         <v>1.6</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="6" t="n">
         <v>99.7</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="3" t="n">
         <v>0.13</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="3" t="n">
         <v>0.08</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="7" t="n">
         <v>0.32</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="7" t="n">
         <v>2.3</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="6" t="n">
         <v>99.40000000000001</v>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="3" t="n">
         <v>0.18</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="3" t="n">
         <v>0.1</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="7" t="n">
         <v>0.38</v>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="7" t="n">
         <v>0.9</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>30 °C/65% RH</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="6" t="n">
         <v>99.2</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="3" t="n">
         <v>0.2</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="3" t="n">
         <v>0.11</v>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F16" s="7" t="n">
         <v>0.46</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G16" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>40 °C/75% RH</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="6" t="n">
         <v>100.2</v>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D17" s="3" t="n">
         <v>0.05</v>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>&lt;0.05</t>
         </is>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F17" s="7" t="n">
         <v>0.17</v>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G17" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>40 °C/75% RH</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="6" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="3" t="n">
         <v>0.09</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="3" t="n">
         <v>0.05</v>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F18" s="7" t="n">
         <v>0.23</v>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="7" t="n">
         <v>2.3</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>40 °C/75% RH</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="6" t="n">
         <v>99.3</v>
       </c>
-      <c r="D19" s="2" t="n">
+      <c r="D19" s="3" t="n">
         <v>0.21</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="3" t="n">
         <v>0.12</v>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="F19" s="7" t="n">
         <v>0.42</v>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G19" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>40 °C/75% RH</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C20" s="6" t="n">
         <v>99.2</v>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="3" t="n">
         <v>0.35</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="3" t="n">
         <v>0.21</v>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F20" s="7" t="n">
         <v>0.66</v>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G20" s="7" t="n">
         <v>2.3</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Complies</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="C21" s="7" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="F21" s="9" t="n"/>
+      <c r="G21" s="9" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>Specification: assay 95.0-105.0% LC; Imp A (RRT 0.86, specified) ≤0.50%; Imp B (RRT 1.12, specified) ≤0.30%; any unspecified impurity ≤0.20%; total impurities ≤2.0%</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n"/>
-      <c r="F22" s="8" t="n"/>
-      <c r="G22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n"/>
     </row>
     <row r="23">
-      <c r="C23" s="7" t="n"/>
-      <c r="F23" s="8" t="n"/>
-      <c r="G23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n"/>
     </row>
     <row r="24">
-      <c r="C24" s="7" t="n"/>
-      <c r="F24" s="8" t="n"/>
-      <c r="G24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9" t="n"/>
     </row>
     <row r="25">
-      <c r="C25" s="7" t="n"/>
-      <c r="F25" s="8" t="n"/>
-      <c r="G25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="9" t="n"/>
     </row>
     <row r="26">
-      <c r="C26" s="7" t="n"/>
-      <c r="F26" s="8" t="n"/>
-      <c r="G26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
     </row>
     <row r="27">
-      <c r="C27" s="7" t="n"/>
-      <c r="F27" s="8" t="n"/>
-      <c r="G27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="F27" s="9" t="n"/>
+      <c r="G27" s="9" t="n"/>
     </row>
     <row r="28">
-      <c r="C28" s="7" t="n"/>
-      <c r="F28" s="8" t="n"/>
-      <c r="G28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="F28" s="9" t="n"/>
+      <c r="G28" s="9" t="n"/>
     </row>
     <row r="29">
-      <c r="C29" s="7" t="n"/>
-      <c r="F29" s="8" t="n"/>
-      <c r="G29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
     </row>
     <row r="30">
-      <c r="C30" s="7" t="n"/>
-      <c r="F30" s="8" t="n"/>
-      <c r="G30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="F30" s="9" t="n"/>
+      <c r="G30" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1319,14 +1326,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Assay and related-substances validation: summary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Validation run under the HPLC method qualification protocol. Acceptance limits as stated in the validation plan.</t>
         </is>
@@ -1334,139 +1341,139 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Acceptance</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Linearity (r²)</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>0.9993</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>≥0.999</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Range (% nominal)</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>50-150</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>80-120 minimum</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Accuracy 80% (% recovery)</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>99.2</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>98.0-102.0</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Accuracy 100% (% recovery)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>100.1</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>98.0-102.0</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Accuracy 120% (% recovery)</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>100.6</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>98.0-102.0</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Repeatability (%RSD, n=6)</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>0.34</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>≤2.0</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Intermediate precision (%RSD)</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>1.22</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>≤2.0</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>LOQ (% of nominal)</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <v>0.05</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>≤0.05</t>
         </is>
@@ -1497,117 +1504,67 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Deviation and sign-off record</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Project disposition and review record</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Record</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Late-eluting peak assigned to impurity reference, no change to method</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Saira Mahmood</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>14/06/2022</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Late-eluting peak</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Resolved against an impurity reference; refer to the identification and integration records.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Capsule formulation retained for transfer</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Alice Penrose</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>30/09/2022</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Capsule formulation</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Retained by Parvessune for transfer.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Interim review of 6-month pulls</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Leon Wu</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Interim review</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>31/03/2022</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Final results and this workbook</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Leon Wu</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Issued Rev03</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>30/09/2022</t>
         </is>

</xml_diff>